<commit_message>
Add broad neuron markers to subtypes
</commit_message>
<xml_diff>
--- a/processed-data/04_snRNA-seq/00_lit_marker_genes/scTypeDB_PEC_PFC_custom.xlsx
+++ b/processed-data/04_snRNA-seq/00_lit_marker_genes/scTypeDB_PEC_PFC_custom.xlsx
@@ -351,26 +351,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>cell_type_broad</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>tissueType</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>cellName</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>geneSymbolmore1</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>geneSymbolmore2</t>
         </is>
@@ -379,540 +384,625 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Astro</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Brain</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Astro</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>ADGRV1,RNF219-AS1,SLC1A3,GFAP,LOC101927437,PTGDS,FBXL7,LINC00499,NHSL1,LRIG1,CDH20,CST3,ATP1A2,AQP4,COL5A3,MT2A,BMPR1B,GRAMD3,DAAM2,FAM189A2,PARD3B,ATP13A4,FGFR3,ZFP36L1,LOC105376244,APOE,LOC101928394,PAMR1,TNC,SLC25A18,ACSS1,PPAP2B,HIF3A,RANBP3L,GLI3,MRVI1,SLC14A1,SLC7A11,ID4,PPP1R3C,ID3,PRODH,NDRG2,ETNPPL,STON2,ITPKB,PON2,ANGPTL4,FOS,PRDM16,ACSBG1,ZFHX4,ACSS3,SLCO1C1,GJA1,HEPACAM,EZR,EYA2,AGT,LAMA1,CDC14A,F3,LOC101926964,LOC101930275,RFTN2,PAPLN,PDK4,YAP1,LOC101927199,S100B,EFEMP1,ALDH1L1,AASS,SOX9,APCDD1,LOC102724289,LOC105376387,MAML2,EYA1,KANK1,GLIS3,LOC105376917,ARHGEF26,GPC5,MMD2,AMZ2,MEGF10,ADGRA3,MEIS2,MSI2,GLUL,ACACB,LINC00609,FOXO1,RAPGEF3,NTM,RFX4,DTNA,SPON1,DOCK1,ARHGAP31,SLC1A2,WDR49,HES1,PREX2,PITPNC1,CACHD1,STK33,NFIA,LINC00299,GPM6A,TSC22D4,PDLIM5,NKAIN3,RGS20,PTPRZ1,MACF1,ZBTB20,NCKAP5,ZNRF3,TRPS1,TNIK,C1orf61,AHCYL2,FGFR2,SLC4A4,LOC105375405,ABLIM1,SLC16A9,NPL,SORBS1,CTNNA2,RFX2,MERTK,SPARCL1,PARD3,ID2,TTYH1,RGMA,PHF21B,QKI,TCF7L2,LIFR,ITPR2,ZHX2,WWOX,CAMK2G,GRAMD1C,NEBL,CSGALNACT1,RYR3,DCLK2,JUN,ADD3,NPAS3,ARHGEF26-AS1,MT3,ACOT11,SFXN5,FNBP1,PRRX1,GNA14,PRKCA,ARHGEF4,KCNN3,OPHN1,SLC39A11,PRKG1,SOX5,GPM6B,NEAT1,ZHX3,PSD2,MYO10,GLUD1,LRRC16A,ARHGAP24,FYN,CRB1,LOC101927335,RORB,CLU,LOC105378763,SCARA3,TPD52L1,PHLPP1,CPE,SHROOM3,VCAN,AHCYL1,SASH1,DDIT4,NCAN,LINC00673,DOCK7,CKB,JUNB,ZSWIM6,PTN,TJP2,OGFRL1,LOC105370983,BMP2K,FGD4,MTSS1L,PFKFB2,ANKDD1A,TPCN1,RHOBTB3,HIP1R,DDAH1,DPP10,TRPM3,CRYAB,EPHB1,IQCA1,HPSE2,TAB2,LINC01411,CABLES1,H3F3B</t>
         </is>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Endo</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Brain</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Endo</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>CLDN5,EPAS1,FLI1,ABCG2,LEF1,EBF1,CGNL1,ID1,HLA-E,IFI27,XAF1,CLEC3B,SLCO1A2,SLCO2B1,ID3,ENG,VIM,LIMS2,EMCN,ZNF366,NOSTRIN,IFI44L,SRGN,SDPR,SLC38A5,IFITM3,TIE1,CXorf36,TGM2,TNFSF10,ROBO4,IFITM1,CD34,GIMAP7,TM4SF18,SOX18,ANO2,PRKCH,ITIH5,IGFBP7,TGFBR2,ANXA3,ATP10A,ADGRL4,PALMD,AIF1L,CLEC14A,KLF2,ITM2A,MFSD2A,FLT1,FLVCR2,SP100,EMP2,SMAD6,UACA,BTNL9,MT2A,ADGRF5,RAMP2,IFI44,ITGA6,HLA-B,LMO2,SLC2A1,VWF,HERC2P3,TMEM204,SLC19A3,RNASE1,C22orf34,A2M,ST8SIA6,ESAM,CFH,CLIC4,PARP14,MECOM,COBLL1,PODXL,ERG,PON2,PAQR5,SHROOM4,PARP9,ARHGAP31,PECAM1,KANK3,NKD1,SH3BP4,TRPM6,INPP5D,HEG1,ALPL,THSD4,NET1,RGCC,PGM5,HMCN1,ABCB1,SLC39A8,HLA-C,B2M,IRAK3,STOM,SLC7A5,APCDD1,WWTR1,ELOVL7,GPCPD1,TMEM123,EGFL7,EPSTI1,ST6GALNAC3,PLEKHG1,HERC2P2,RCSD1,CFLAR,DOCK1,TANC1,HERC2P9,C10orf11,APOLD1,SYNE2,PTPRG,NXN,HIF3A,DUSP1,MYO10,SLC7A1,PTPRB,CYYR1,NEAT1,ESYT2,ST6GAL1,IGF1R,NPIPB4,TNS1,CDC14A,SLC39A10,TACC1,UTRN,GPR85,HSPA1B,PROM1,SGMS1,ARHGAP29,ENTPD1,CA4,MYO1E,DOCK9,PPFIBP1,GALNT15,PREX2,TEK,FAXDC2,PTPN14,MSN,SLC7A11,NFKBIA,LOC101928570,LHFP,PRTG,TMEM2,TBC1D4,LDLRAD3,SPTBN1,RNF144B,KIAA1462,ADIPOR2,CMAHP,FN1,HLA-A,SERPINB6,RIN2,TJP1,FMNL3,ELF1,ITGA1,EPB41L4A,ETS1,RAPGEF2,FOXO1,DACH1,AFAP1L2,PDLIM5,MTUS1,GALNT18,SLC9A3R2,FOXP1,APBB2,MEF2A,ZBTB20,NRP1,BSG,HSPA1A,ETS2,LAMA3,RBMS2,CLIC5,CD320,USP54,BBS9,RBMS3,SNED1,SEC14L1,ACVR1,FRYL,HERPUD1,CTBP2,TNS2,RBM20,TFRC,LAMA4,LINC00472,USP6NL,PDXK,RASSF3,CCNY,KANK1,BMPR2,TIMP3,CTNNB1,PPARD,DLEU2,UNC13B,LOC102467224,TMSB10,CCND3,RUNDC3B,ANKS1A,JAM2,RNR2,CRIM1,IFNAR2,SLC7A5P2,AGFG1,GSN,NRP2,LEPR,JUN,MX1,SDCBP,NAMPT,MYH9,STK3,PLA2G4A,USP53,SPOCK2,GNAI2,LMBR1,LRRC8C,ACTN4,UBC,AFF1,IFNGR1,LOC105370526,GAB1,FGD6,LY6E,RHOBTB1,SCARB1,KLF6,SLC5A6,CDYL2,HLF,PIK3R3,SHANK3,PLCB4,SLC1A1,SGPP2,RASSF8,ATP6,EEF1A1,RAPGEF1,IQGAP1,PARD3B,H3F3B,BMP6,IKBKB,ND4,PPAP2A,TDRP,CYTB,HIPK3,ARHGEF10,RAD51B</t>
         </is>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Excit</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Excit</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SLC17A7,SATB2,SV2B</t>
-        </is>
-      </c>
-      <c r="D4">
+          <t>Excit.L2_3_IT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SLC17A7,SATB2,SV2B,CA10,FAM19A1,LAMA2,PTPRK,CUX2,KCNIP4,LOC101927745,CBLN2,LDB2,COL5A2,LOC101928964,LOC105378334,CADPS2</t>
+        </is>
+      </c>
+      <c r="E4">
         <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Excit</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Excit.L2_3_IT</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CA10,FAM19A1,LAMA2,PTPRK,CUX2,KCNIP4,LOC101927745,CBLN2,LDB2,COL5A2,LOC101928964,LOC105378334,CADPS2</t>
-        </is>
-      </c>
-      <c r="D5">
+          <t>Excit.L4_IT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SLC17A7,SATB2,SV2B,RORB,RMST,POU6F2,CPNE4,TSHZ2,OTOGL,LINCR-0002,LOC105371832,FSTL4,DCC,IL1RAPL2,LOC100132891,LOC105373893,PTPRD,SCHLAP1,FAM19A1,LOC105374971,PLCH1</t>
+        </is>
+      </c>
+      <c r="E5">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Excit</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Excit.L4_IT</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>RORB,RMST,POU6F2,CPNE4,TSHZ2,OTOGL,LINCR-0002,LOC105371832,FSTL4,DCC,IL1RAPL2,LOC100132891,LOC105373893,PTPRD,SCHLAP1,FAM19A1,LOC105374971,PLCH1</t>
-        </is>
-      </c>
-      <c r="D6">
+          <t>Excit.L5_6_NP</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SLC17A7,SATB2,SV2B,HTR2C,TSHZ2,NPSR1-AS1,LOC729732,HS3ST4,ITGA8,ASIC2,SORCS2,LOC105378334,LOC101928095,TLE4,CHN2,CDH6,TLL1,GRM8,LOC101928948,CRYM,LOC101928114,COL12A1,OLFM3,CPNE4,LOC645544,TOX,SEMA3E,NXPH2,SEMA5B,LOC105369818,KIAA1456,GRM3,DPY19L1,DIRAS2,GHR,MPP7,NPSR1,ZNF385D,ETV1,LDB2,FER1L6-AS2,LOC100506457,PCP4,FOXP2,DOCK4,LY86-AS1,ATP2C2,FGFR1,CLSTN2,KCTD8,CD36,SPON1,LOC100130459,CHRM2,ADAMTSL1,GPC5</t>
+        </is>
+      </c>
+      <c r="E6">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Excit</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Excit.L5_6_NP</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>HTR2C,TSHZ2,NPSR1-AS1,LOC729732,HS3ST4,ITGA8,ASIC2,SORCS2,LOC105378334,LOC101928095,TLE4,CHN2,CDH6,TLL1,GRM8,LOC101928948,CRYM,LOC101928114,COL12A1,OLFM3,CPNE4,LOC645544,TOX,SEMA3E,NXPH2,SEMA5B,LOC105369818,KIAA1456,GRM3,DPY19L1,DIRAS2,GHR,MPP7,NPSR1,ZNF385D,ETV1,LDB2,FER1L6-AS2,LOC100506457,PCP4,FOXP2,DOCK4,LY86-AS1,ATP2C2,FGFR1,CLSTN2,KCTD8,CD36,SPON1,LOC100130459,CHRM2,ADAMTSL1,GPC5</t>
-        </is>
-      </c>
-      <c r="D7">
+          <t>Excit.L5_ET</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SLC17A7,SATB2,SV2B,FAM19A1,LOC101927745,COL24A1,COL5A2,LOC105378657,VAT1L,NRP1,PCSK6,CBLN2,PTCHD1-AS,CLEC2L,CABP1,KCNN2,LMO7,HOMER1,ESRRG,GRM8,NRGN,NRG1,PEX5L,TOX,SLC35F3,KCNIP4,LOC101928923</t>
+        </is>
+      </c>
+      <c r="E7">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Excit</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Excit.L5_ET</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>FAM19A1,LOC101927745,COL24A1,COL5A2,LOC105378657,VAT1L,NRP1,PCSK6,CBLN2,PTCHD1-AS,CLEC2L,CABP1,KCNN2,LMO7,HOMER1,ESRRG,GRM8,NRGN,NRG1,PEX5L,TOX,SLC35F3,KCNIP4,LOC101928923</t>
-        </is>
-      </c>
-      <c r="D8">
+          <t>Excit.L5_IT</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>SLC17A7,SATB2,SV2B,LOC105374971,CPNE4,IL1RAPL2,CADPS2,RORB,TOX,FOXP2,RXFP1,LOC105373893,FSTL4,EPHA3,POU6F2,PTPRK,LOC401134,CLSTN2,HS3ST2,ARHGAP15,KCNIP4,PDZRN4</t>
+        </is>
+      </c>
+      <c r="E8">
         <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Excit</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Excit.L5_IT</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LOC105374971,CPNE4,IL1RAPL2,CADPS2,RORB,TOX,FOXP2,RXFP1,LOC105373893,FSTL4,EPHA3,POU6F2,PTPRK,LOC401134,CLSTN2,HS3ST2,ARHGAP15,KCNIP4,PDZRN4</t>
-        </is>
-      </c>
-      <c r="D9">
+          <t>Excit.L6_CT</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SLC17A7,SATB2,SV2B,LOC105371833,SEMA3E,LOC105373592,MEIS2,ADAMTSL1,LOC105373893,HS3ST4,TRPM3,FOXP2,SEMA5A,EGFEM1P,TLE4,COL24A1,LOC401478,DLC1,ASIC2,PDZRN4,SV2B,RALYL,RYR3,PEX5L,LDB2,ZFPM2,PDE1A,CLSTN2</t>
+        </is>
+      </c>
+      <c r="E9">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Excit</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Excit.L6_CT</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LOC105371833,SEMA3E,LOC105373592,MEIS2,ADAMTSL1,LOC105373893,HS3ST4,TRPM3,FOXP2,SEMA5A,EGFEM1P,TLE4,COL24A1,LOC401478,DLC1,ASIC2,PDZRN4,SV2B,RALYL,RYR3,PEX5L,LDB2,ZFPM2,PDE1A,CLSTN2</t>
-        </is>
-      </c>
-      <c r="D10">
+          <t>Excit.L6_IT</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SLC17A7,SATB2,SV2B,LOC105373893,CBLN2,LOC284930,LOC105371832,SLIT3,PTPRK,LOC101928964</t>
+        </is>
+      </c>
+      <c r="E10">
         <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Excit</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Excit.L6_IT</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LOC105373893,CBLN2,LOC284930,LOC105371832,SLIT3,PTPRK,LOC101928964</t>
-        </is>
-      </c>
-      <c r="D11">
+          <t>Excit.L6_IT_Car3</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>SLC17A7,SATB2,SV2B,NTNG2,THEMIS,LOC105378486,MCTP2,SNTB1,ITGB8,LOC105370983,GSG1L,NWD2,CADPS2,TRPC5,CA10,DACH1,SATB2,KCNIP4,ZNF804B,ERC2,PDE1A,ARAP2,SORBS2,CUX1,KCTD16,CLSTN2,LOC101928964,TMEM132D,UNC5C,MGAT5,AK5,RIT2,PDZRN4,TENM4,GALNT14,RGS12,SPOCK1,PCDH9,NRG1,FRAS1,CPNE4,CTNNA3,LOC105371308</t>
+        </is>
+      </c>
+      <c r="E11">
         <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Excit</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Excit.L6_IT_Car3</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>NTNG2,THEMIS,LOC105378486,MCTP2,SNTB1,ITGB8,LOC105370983,GSG1L,NWD2,CADPS2,TRPC5,CA10,DACH1,SATB2,KCNIP4,ZNF804B,ERC2,PDE1A,ARAP2,SORBS2,CUX1,KCTD16,CLSTN2,LOC101928964,TMEM132D,UNC5C,MGAT5,AK5,RIT2,PDZRN4,TENM4,GALNT14,RGS12,SPOCK1,PCDH9,NRG1,FRAS1,CPNE4,CTNNA3,LOC105371308</t>
-        </is>
-      </c>
-      <c r="D12">
+          <t>Excit.L6b</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>SLC17A7,SATB2,SV2B,HS3ST4,TLE4,MARCH1,ZFHX3,LOC401134,PDZRN4,NFIA,ARPP21,DLC1,SEMA3A,MDFIC,KIAA1217,SLIT3,ZFPM2,PCSK5,LMO3,RXFP1,DPYD,MLIP,C10orf11,FUT9,FOXP2,MEIS2,CDH10,ZBTB7C,RALYL,CELF2,LOC100132891,PTPRD,DGKG</t>
+        </is>
+      </c>
+      <c r="E12">
         <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Inhib</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Excit.L6b</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>HS3ST4,TLE4,MARCH1,ZFHX3,LOC401134,PDZRN4,NFIA,ARPP21,DLC1,SEMA3A,MDFIC,KIAA1217,SLIT3,ZFPM2,PCSK5,LMO3,RXFP1,DPYD,MLIP,C10orf11,FUT9,FOXP2,MEIS2,CDH10,ZBTB7C,RALYL,CELF2,LOC100132891,PTPRD,DGKG</t>
-        </is>
-      </c>
-      <c r="D13">
+          <t>Inhib.Chandelier</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>GAD1,GAD2,CA8,NPNT,FAM19A4,UNC5B,ZNF385D-AS2,LOC101928964,SLC9A9,TRPS1,HPSE2,DPP10-AS3,RORA,ZNF385D,GULP1,CNTN5,PLCXD3,DPP10,CALN1,ALK,RASSF8,TMEM132C,MIR4500HG,DLGAP2,CNTNAP3B,SRGAP1,LHFPL3,MYO16,SDK1,TMEM132D,HTR1F,TENM1,THSD7A,TENM4,ANK1,ADAMTS17,SGCD,ZNF536,KCNAB1,EDIL3,ADCY8,ZNF804A,LOC102724790,FAM19A2</t>
+        </is>
+      </c>
+      <c r="E13">
         <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Inhib</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Inhib</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GAD1,GAD2</t>
-        </is>
-      </c>
-      <c r="D14">
+          <t>Inhib.Lamp5</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>GAD1,GAD2,RELN,LINC00299,PRELID2,CXCL14,FGF13,HS3ST5,SV2C,MYO16,TRPC3,FREM1,CACNA2D1,GAD2,DOCK10,EGFR,ADARB2,FSTL5,KIT,PTCHD4,SLC6A1,DNER,NYAP2,LOC101927870,CNTNAP4,SGCZ,EYA4,FBXL7,ALK,INPP4B,NRG1,COL5A2</t>
+        </is>
+      </c>
+      <c r="E14">
         <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Inhib</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Inhib.Chandelier</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CA8,NPNT,FAM19A4,UNC5B,ZNF385D-AS2,LOC101928964,SLC9A9,TRPS1,HPSE2,DPP10-AS3,RORA,ZNF385D,GULP1,CNTN5,PLCXD3,DPP10,CALN1,ALK,RASSF8,TMEM132C,MIR4500HG,DLGAP2,CNTNAP3B,SRGAP1,LHFPL3,MYO16,SDK1,TMEM132D,HTR1F,TENM1,THSD7A,TENM4,ANK1,ADAMTS17,SGCD,ZNF536,KCNAB1,EDIL3,ADCY8,ZNF804A,LOC102724790,FAM19A2</t>
-        </is>
-      </c>
-      <c r="D15">
+          <t>Inhib.Lamp5_Lhx6</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>GAD1,GAD2,FGF13,PDGFD,EYA4,NTNG1,CHST9,FBXL7,MYO16,UNC5D,GRIA4,TOX,SV2C,LAMP5,LTBP1,LINC00403,LINC00299,VAV3,NOS1,CA1,CA8,LOC105371641,KIT,SFRP1,COL4A2,LINC01314,TACR1,GAD2,CDHR3,CACNA2D1,SPHKAP,ALK,IGSF11,RAB3IP,PTCHD4,GRIN2A,SLC6A1,UNC13C,ZNF536,PTPRT,GRIP1,NFIB,EGFEM1P,SEMA6D,KIRREL3,MGAT4C,PRELID2,MYRFL,SGCZ,SOX2-OT,NKAIN3,FSTL5</t>
+        </is>
+      </c>
+      <c r="E15">
         <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Inhib</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Inhib.Lamp5</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>RELN,LINC00299,PRELID2,CXCL14,FGF13,HS3ST5,SV2C,MYO16,TRPC3,FREM1,CACNA2D1,GAD2,DOCK10,EGFR,ADARB2,FSTL5,KIT,PTCHD4,SLC6A1,DNER,NYAP2,LOC101927870,CNTNAP4,SGCZ,EYA4,FBXL7,ALK,INPP4B,NRG1,COL5A2</t>
-        </is>
-      </c>
-      <c r="D16">
+          <t>Inhib.Pax6</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>GAD1,GAD2,CXCL14,SORCS3,ADARB2,SLC35F4,MAML3,RELN,MYO16,CNR1,RBMS3,SGCD,PBX3,CHRNA7,DDR2,SHISA9,B3GALT1,CDH4,CCK,ZNF385D,CCDC85A,IL1RAPL2,PLCXD3,ALK,YJEFN3</t>
+        </is>
+      </c>
+      <c r="E16">
         <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Inhib</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Inhib.Lamp5_Lhx6</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>FGF13,PDGFD,EYA4,NTNG1,CHST9,FBXL7,MYO16,UNC5D,GRIA4,TOX,SV2C,LAMP5,LTBP1,LINC00403,LINC00299,VAV3,NOS1,CA1,CA8,LOC105371641,KIT,SFRP1,COL4A2,LINC01314,TACR1,GAD2,CDHR3,CACNA2D1,SPHKAP,ALK,IGSF11,RAB3IP,PTCHD4,GRIN2A,SLC6A1,UNC13C,ZNF536,PTPRT,GRIP1,NFIB,EGFEM1P,SEMA6D,KIRREL3,MGAT4C,PRELID2,MYRFL,SGCZ,SOX2-OT,NKAIN3,FSTL5</t>
-        </is>
-      </c>
-      <c r="D17">
+          <t>Inhib.Pvalb</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>GAD1,GAD2,SLIT2,PPARGC1A,ADAMTS17,NXPH1,KCNC2,ERBB4,BTBD11,MYO5B,TMEM132C,ZNF804A,PRKG1,DPP10</t>
+        </is>
+      </c>
+      <c r="E17">
         <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Inhib</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Inhib.Pax6</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CXCL14,SORCS3,ADARB2,SLC35F4,MAML3,RELN,MYO16,CNR1,RBMS3,SGCD,PBX3,CHRNA7,DDR2,SHISA9,B3GALT1,CDH4,CCK,ZNF385D,CCDC85A,IL1RAPL2,PLCXD3,ALK,YJEFN3</t>
-        </is>
-      </c>
-      <c r="D18">
+          <t>Inhib.Sncg</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>GAD1,GAD2,CXCL14,CNR1,PRELID2,CNTN5,FSTL5,ADARB2,CNTNAP4,INPP4B,CHRNA7,RGS12,NR2F2-AS1,NPAS3,ADRA1A,IL1RAPL2,THSD7B,CCK,SORCS1,CDH4</t>
+        </is>
+      </c>
+      <c r="E18">
         <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Inhib</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Inhib.Pvalb</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SLIT2,PPARGC1A,ADAMTS17,NXPH1,KCNC2,ERBB4,BTBD11,MYO5B,TMEM132C,ZNF804A,PRKG1,DPP10</t>
-        </is>
-      </c>
-      <c r="D19">
+          <t>Inhib.Sst</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>GAD1,GAD2,GRIK1,TRHDE,SST,NXPH1,STXBP6,COL25A1,SPOCK3,KIF26B,SOX6,KIAA1217,GRIN3A,WLS,LOC105377567,CDH9,PLCH1,GRIK3,ST6GALNAC5,XKR4,SHISA6</t>
+        </is>
+      </c>
+      <c r="E19">
         <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Inhib</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Inhib.Sncg</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CXCL14,CNR1,PRELID2,CNTN5,FSTL5,ADARB2,CNTNAP4,INPP4B,CHRNA7,RGS12,NR2F2-AS1,NPAS3,ADRA1A,IL1RAPL2,THSD7B,CCK,SORCS1,CDH4</t>
-        </is>
-      </c>
-      <c r="D20">
+          <t>Inhib.Sst_Chodl</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>GAD1,GAD2,NPY,CRHBP,NOS1,SST,TACR1,TRPC6,SOX6,CCDC109B,ARHGAP24,IL1RAPL2,COL24A1,GULP1,MPPED2,NXPH2,LRP8,LARGE,GRIK1,TMTC1,RPS6KA2,FRMD4B,DGKG,SOX2-OT,THSD4,NELL1,TAC1,NNAT</t>
+        </is>
+      </c>
+      <c r="E20">
         <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Inhib</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Inhib.Sst</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GRIK1,TRHDE,SST,NXPH1,STXBP6,COL25A1,SPOCK3,KIF26B,SOX6,KIAA1217,GRIN3A,WLS,LOC105377567,CDH9,PLCH1,GRIK3,ST6GALNAC5,XKR4,SHISA6</t>
-        </is>
-      </c>
-      <c r="D21">
+          <t>Inhib.Vip</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>GAD1,GAD2,VIP,ADARB2,GALNTL6,THSD7A,RGS12,TAC3,SCG2,PLD5,ZBTB20,LOC105373642,PROX1,ERBB4,GALNT13,SHISA8,DLX6-AS1,SLC24A3,SYNPR,EGFEM1P,THSD7B</t>
+        </is>
+      </c>
+      <c r="E21">
         <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Micro</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Inhib.Sst_Chodl</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>NPY,CRHBP,NOS1,SST,TACR1,TRPC6,SOX6,CCDC109B,ARHGAP24,IL1RAPL2,COL24A1,GULP1,MPPED2,NXPH2,LRP8,LARGE,GRIK1,TMTC1,RPS6KA2,FRMD4B,DGKG,SOX2-OT,THSD4,NELL1,TAC1,NNAT</t>
-        </is>
-      </c>
-      <c r="D22">
+          <t>Micro</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>DOCK8,APBB1IP,TBXAS1,ZFP36L2,SLCO2B1,CSF1R,C3,FYB,LOC101929497,CX3CR1,SYK,SAMSN1,IKZF1,PTPRC,FAM177B,CD74,RHBDF2,PIK3R5,FLI1,FGD2,TMEM156,RGS10,P2RY13,ITGAX,MS4A7,CSF3R,C10orf54,LINC00996,CD86,CYBA,C1QB,LINC01268,TAL1,LOC105376604,LOC105372984,HLA-DRA,LST1,LOC105376388,CLEC7A,INPP5D,WDFY4,TLR2,ADAM28,LPAR6,NCKAP1L,SP100,LPAR5,P2RY12,BLNK,TGFBR2,PLCG2,LAPTM5,CSF2RA,LOC105377594,ZFP36L1,OLR1,RUNX1,IRF8,SLC1A3,LYN,CD53,CYBB,BNC2,TFEC,C10orf11,IL13RA1,AOAH,LOC105377918,LY86,MILR1,LOC105378305,NFATC2,CYTH4,PALD1,ARHGAP24,RREB1,IFI16,RBM47,ITGAM,LINC01141,BIN2,ALOX5,A2M,SLC2A5,PLXDC2,MERTK,LOC105369290,RCSD1,MRC1,ZFHX3,ADAP2,ENTPD1,LPCAT2,GPR34,CPED1,ST6GAL1,LTC4S,LOC105370359,SFMBT2,PIK3AP1,ARRDC5,TMIGD3,LOC105377684,AXL,DOCK2,ITPR2,DOCK4,MAML2,GGTA1P,MEF2A,ABCC4,ARHGAP15,ELMO1,ATP8B4,AKAP13,IPCEF1,FOXN3,CYFIP1,HCK,FRMD4A,ARHGAP22,SORL1,PREX1,HS3ST4,TNS3,SRGAP2,S100Z,SLC9A9,IRAK3,MAML3,LOC101930023,EPB41L2,ST6GALNAC3,QKI,LDLRAD4,MYO1F,PARP14,FMNL3,SYNDIG1,ARHGAP25,ANKRD44,RASGEF1C,DIAPH2,LRRK1,LHFPL2,CIITA,MEF2C,SPP1,CARD11,MED13L,CHST11,MYOF,MBNL1,VAV1,MAP4K4,SRGAP2B,KCNQ3,IGSF10,APOE,TGFBR1,PGM5,BMP2K,TBC1D22A,ZNF710,HAVCR2,NRROS,PLA2G4A,C12orf75,FOXP2,FCHSD2,ATM,ZSWIM6,PICALM,FAM105A,CSGALNACT1,RNASET2,LPAR1,WIPF1,RIN3,DLEU7-AS1,IL18,LOC101929294,B3GNT5,USP53,SNX29,RYR1,TCF12,HSPA1B,ZFPM2-AS1,LOC401134,ELF1,IL6ST,TGFB1,LOC105376819,NEAT1,MGAT4A,MRC2,CAPZB,ADGRG1,DOCK10,ETV6,SOCS6,WASF2,HTRA1,NCKAP5,PTPRJ,BHLHE41,NPL,DIP2B,IFNGR1,DLEU2,MIS18BP1,CHD7,KCNK13,RAD51B,MAP3K5,AFF1,CTBP2,SRGAP2C,KIAA0226L,FGD4,SMAP2,ITM2B,ABR,ITGB5,SIPA1L2,CECR2,FKBP5,B2M,RAB31,SPRED1,IL17RA,DENND3,MCF2L,USP6NL,GAB2,SRGAP2-AS1,MTHFD1L,DISP1,HSPA1A,RAPGEF1,SPI1,SAT1,MARCH3,SLC4A7,PLD1,SKAP2,MIR31HG,LOC105372874,RUNX2,ARHGAP12,AP1B1,SH3KBP1,GNG7,PRDM11,MKNK1,SUSD6,LRCH1,CFLAR,PAG1,TBC1D12,GSN,LOC105377632,NLRP1,APPL2,TAB2,SRGAP1,NRIP1,KBTBD12,UBE2E1,ARHGEF6,SERPINB9,SH2B3,RAP1A,SETX,KCNQ1,ZNRF2,ARHGAP6,ENTPD1-AS1,IGSF21,MANBA,LRRC8C,RNF213,BCAR3,RASSF8</t>
+        </is>
+      </c>
+      <c r="E22">
         <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>OPC</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Inhib.Vip</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>VIP,ADARB2,GALNTL6,THSD7A,RGS12,TAC3,SCG2,PLD5,ZBTB20,LOC105373642,PROX1,ERBB4,GALNT13,SHISA8,DLX6-AS1,SLC24A3,SYNPR,EGFEM1P,THSD7B</t>
-        </is>
-      </c>
-      <c r="D23">
+          <t>OPC</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>PDGFRA,BCAS1,OLIG1,ZCCHC24,LOC105374875,OLIG2,PLLP,APOD,C5orf64,LOC105379054,SHROOM4,VCAN,C10orf90,RFTN2,SMOC1,FERMT1,ATP10B,DOCK1,LOC105377632,MAML2,COL9A1,BCAN,PTPRZ1,MEGF11,KCNH8,PCDH15,PLEKHH2,LHFPL3,CA10,TNS3,STK32A,SEMA5A,TNR,LINC00673,SOX6,PTN,CHD7,DSCAM,ARHGAP31,EPN2,XYLT1,ZFHX4,MYT1,LRRC4C,OPHN1,AGAP1,SPATA6,KAT2B,PRRX1,SCD5,LUZP2,LDLRAD3,NOVA1,LOC102725045,APBB2,CHST11,KIF13A,ATP13A4,NCKAP5,DGKG,NTN1,KANK1,SULF2,CDH20,BRINP3,PDZD2,NTNG1,QKI,DPP6,MMP16,ZSWIM6,SLC35F1,LRRN1,ZNF462,NTM,ZBTB20,COL11A1,LOC100506457,PHLPP1,NAV1,NFIA,C10orf11,LOC105378311,C1orf61,NLGN4Y,USP24,LPPR1,KLHL1,MMD2,HIP1,PDE4B,RAB31,TMEM132C,PEAK1,HTRA1,ADAMTS17,LOC101927293,ABHD2,KCNMB2,ITPR2,MPPED2,SEZ6L,ZFPM2,PREX2,HIP1R,CMYA5,NKAIN3,TNK2,ZEB1,TMEM163,UST,CASK,LMF1,SH3D19,RIN2,ZHX2,PID1,TCF7L2,GALNT10,KCNMB2-AS1,SERINC5,IPO9-AS1</t>
+        </is>
+      </c>
+      <c r="E23">
         <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Oligo</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Micro</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DOCK8,APBB1IP,TBXAS1,ZFP36L2,SLCO2B1,CSF1R,C3,FYB,LOC101929497,CX3CR1,SYK,SAMSN1,IKZF1,PTPRC,FAM177B,CD74,RHBDF2,PIK3R5,FLI1,FGD2,TMEM156,RGS10,P2RY13,ITGAX,MS4A7,CSF3R,C10orf54,LINC00996,CD86,CYBA,C1QB,LINC01268,TAL1,LOC105376604,LOC105372984,HLA-DRA,LST1,LOC105376388,CLEC7A,INPP5D,WDFY4,TLR2,ADAM28,LPAR6,NCKAP1L,SP100,LPAR5,P2RY12,BLNK,TGFBR2,PLCG2,LAPTM5,CSF2RA,LOC105377594,ZFP36L1,OLR1,RUNX1,IRF8,SLC1A3,LYN,CD53,CYBB,BNC2,TFEC,C10orf11,IL13RA1,AOAH,LOC105377918,LY86,MILR1,LOC105378305,NFATC2,CYTH4,PALD1,ARHGAP24,RREB1,IFI16,RBM47,ITGAM,LINC01141,BIN2,ALOX5,A2M,SLC2A5,PLXDC2,MERTK,LOC105369290,RCSD1,MRC1,ZFHX3,ADAP2,ENTPD1,LPCAT2,GPR34,CPED1,ST6GAL1,LTC4S,LOC105370359,SFMBT2,PIK3AP1,ARRDC5,TMIGD3,LOC105377684,AXL,DOCK2,ITPR2,DOCK4,MAML2,GGTA1P,MEF2A,ABCC4,ARHGAP15,ELMO1,ATP8B4,AKAP13,IPCEF1,FOXN3,CYFIP1,HCK,FRMD4A,ARHGAP22,SORL1,PREX1,HS3ST4,TNS3,SRGAP2,S100Z,SLC9A9,IRAK3,MAML3,LOC101930023,EPB41L2,ST6GALNAC3,QKI,LDLRAD4,MYO1F,PARP14,FMNL3,SYNDIG1,ARHGAP25,ANKRD44,RASGEF1C,DIAPH2,LRRK1,LHFPL2,CIITA,MEF2C,SPP1,CARD11,MED13L,CHST11,MYOF,MBNL1,VAV1,MAP4K4,SRGAP2B,KCNQ3,IGSF10,APOE,TGFBR1,PGM5,BMP2K,TBC1D22A,ZNF710,HAVCR2,NRROS,PLA2G4A,C12orf75,FOXP2,FCHSD2,ATM,ZSWIM6,PICALM,FAM105A,CSGALNACT1,RNASET2,LPAR1,WIPF1,RIN3,DLEU7-AS1,IL18,LOC101929294,B3GNT5,USP53,SNX29,RYR1,TCF12,HSPA1B,ZFPM2-AS1,LOC401134,ELF1,IL6ST,TGFB1,LOC105376819,NEAT1,MGAT4A,MRC2,CAPZB,ADGRG1,DOCK10,ETV6,SOCS6,WASF2,HTRA1,NCKAP5,PTPRJ,BHLHE41,NPL,DIP2B,IFNGR1,DLEU2,MIS18BP1,CHD7,KCNK13,RAD51B,MAP3K5,AFF1,CTBP2,SRGAP2C,KIAA0226L,FGD4,SMAP2,ITM2B,ABR,ITGB5,SIPA1L2,CECR2,FKBP5,B2M,RAB31,SPRED1,IL17RA,DENND3,MCF2L,USP6NL,GAB2,SRGAP2-AS1,MTHFD1L,DISP1,HSPA1A,RAPGEF1,SPI1,SAT1,MARCH3,SLC4A7,PLD1,SKAP2,MIR31HG,LOC105372874,RUNX2,ARHGAP12,AP1B1,SH3KBP1,GNG7,PRDM11,MKNK1,SUSD6,LRCH1,CFLAR,PAG1,TBC1D12,GSN,LOC105377632,NLRP1,APPL2,TAB2,SRGAP1,NRIP1,KBTBD12,UBE2E1,ARHGEF6,SERPINB9,SH2B3,RAP1A,SETX,KCNQ1,ZNRF2,ARHGAP6,ENTPD1-AS1,IGSF21,MANBA,LRRC8C,RNF213,BCAR3,RASSF8</t>
-        </is>
-      </c>
-      <c r="D24">
+          <t>Oligo</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ST18,ENPP2,C10orf90,DOCK5,LOC101927459,MOG,BCAS1,CNDP1,UGT8,LOC101929249,CLDN11,COL4A5,CARNS1,FA2H,ABCA8,SHROOM4,OPALIN,TMEM63A,SLCO1A2,MAG,MYRF,LINC00639,FOLH1,SEPP1,PLLP,TRIM59,SH3TC2,ASPA,RNASE1,MAL,CD9,TMEM235,KIAA1755,PPP1R14A,TMEM98,CD22,ERMN,SEMA3B,PLP1,MOBP,KCNH8,ITGA2,RFTN2,ZCCHC24,TTYH2,CERCAM,CDH19,PRR5L,DAAM2,LOC101927967,PTGDS,LPAR1,SPP1,S100B,LOC100507336,SLC5A11,FAM107B,LOC100130370,ERBB3,TMEM144,ANLN,GPR37,VRK2,PMP22,APOD,RNF220,RGCC,CPM,PLA2G16,HEPACAM,PLD1,LDB3,DOCK1,CLMN,HEPN1,MBP,CNP,CLIC4,LINC00320,LINC00609,PIP4K2A,FRMD4B,CTNNA3,NCKAP5,QKI,CREB5,LINC01170,PLEKHH1,SIK3,LRP2,PPP2R2B,FGFR2,PCDH9,ELMO1,SLC44A1,PHLPP1,PDE4B,SLC24A2,ATP10B,GAB1,SCD,CDK18,DOCK10,PLCL1,PHLDB1,NINJ2,EDIL3,NDE1,MYO1E,IL1RAPL1,GLDN,MAP7,CAPN3,TCF12,SEPT7,TF,FMNL2,FRMD5,CRYAB,PXK,PDE8A,MEGF10,MAN2A1,FBXL7,TMEM165,FRYL,DLG1,DPYD,TTLL7,TMTC2,TRIM2,KIAA1598,GPRC5B,ERBB2IP,ZBTB20,GSN,DNAJC6,PTPRK,GATM,UNC5C,CA2,MAP4K4,ARAP2,PRUNE2,TJP1,HHIP,HAPLN2,CDH20,GPM6B,SYNJ2,USP54,PDE1C,SLAIN1,FUT8,DNM3,CLDND1,GRM3,PCSK6,LAMP2,HIPK2,WIPF1,ABCA2,APBB2,ATP8A1,ENOSF1,EFHD1,AGAP1,PICALM,MBNL2,HIP1,PREX1,SH3GL3,MARCH1,KIF13A,LPGAT1,FAXDC2,CNTN2,TSC22D4,APLP1,ZEB2,PIEZO2,MYO1D,COBL,SMA4,ZFHX4,PTN,FAM124A,ARHGAP21,SCD5,PEX5L,PTBP2,AMER2,MAP4K5,SLCO3A1,DIP2B,SH3D19,ZFYVE16,LANCL1,SORT1,FNBP1,CHD7,LOC101927768,PSEN1,RYBP,CBR1,FTH1,NEAT1,ADIPOR2,QDPR,TULP4,KLHL32,KLHL4,SUN2,CDK19,FAM13C,KIF6,SEMA6A,JAM3,RHOU,LOC100128079,KIF13B,HS3ST5,CHN2,SGK1,MTUS1,SEMA4D,PLXDC2,LOC100287225,PALM2,FOXN2,TESK2,NEO1,MOB3B,TUBA1A,KANK1,ATG4C,MARCKSL1,MVB12B,ACER3,AATK,IQGAP1,CUEDC1,SLC12A2,SLC22A15,CCP110,SECISBP2L,COLGALT2,SLC25A13,LRRC8D,SPATA6,PCDH9-AS2,RAD51B,GNG7,BIN1,YPEL2</t>
+        </is>
+      </c>
+      <c r="E24">
         <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>Tcell</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>OPC</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PDGFRA,BCAS1,OLIG1,ZCCHC24,LOC105374875,OLIG2,PLLP,APOD,C5orf64,LOC105379054,SHROOM4,VCAN,C10orf90,RFTN2,SMOC1,FERMT1,ATP10B,DOCK1,LOC105377632,MAML2,COL9A1,BCAN,PTPRZ1,MEGF11,KCNH8,PCDH15,PLEKHH2,LHFPL3,CA10,TNS3,STK32A,SEMA5A,TNR,LINC00673,SOX6,PTN,CHD7,DSCAM,ARHGAP31,EPN2,XYLT1,ZFHX4,MYT1,LRRC4C,OPHN1,AGAP1,SPATA6,KAT2B,PRRX1,SCD5,LUZP2,LDLRAD3,NOVA1,LOC102725045,APBB2,CHST11,KIF13A,ATP13A4,NCKAP5,DGKG,NTN1,KANK1,SULF2,CDH20,BRINP3,PDZD2,NTNG1,QKI,DPP6,MMP16,ZSWIM6,SLC35F1,LRRN1,ZNF462,NTM,ZBTB20,COL11A1,LOC100506457,PHLPP1,NAV1,NFIA,C10orf11,LOC105378311,C1orf61,NLGN4Y,USP24,LPPR1,KLHL1,MMD2,HIP1,PDE4B,RAB31,TMEM132C,PEAK1,HTRA1,ADAMTS17,LOC101927293,ABHD2,KCNMB2,ITPR2,MPPED2,SEZ6L,ZFPM2,PREX2,HIP1R,CMYA5,NKAIN3,TNK2,ZEB1,TMEM163,UST,CASK,LMF1,SH3D19,RIN2,ZHX2,PID1,TCF7L2,GALNT10,KCNMB2-AS1,SERINC5,IPO9-AS1</t>
-        </is>
-      </c>
-      <c r="D25">
+          <t>Tcell</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ST18,PTPRC</t>
+        </is>
+      </c>
+      <c r="E25">
         <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Brain</t>
+          <t>VLMC</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Oligo</t>
+          <t>Brain</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ST18,ENPP2,C10orf90,DOCK5,LOC101927459,MOG,BCAS1,CNDP1,UGT8,LOC101929249,CLDN11,COL4A5,CARNS1,FA2H,ABCA8,SHROOM4,OPALIN,TMEM63A,SLCO1A2,MAG,MYRF,LINC00639,FOLH1,SEPP1,PLLP,TRIM59,SH3TC2,ASPA,RNASE1,MAL,CD9,TMEM235,KIAA1755,PPP1R14A,TMEM98,CD22,ERMN,SEMA3B,PLP1,MOBP,KCNH8,ITGA2,RFTN2,ZCCHC24,TTYH2,CERCAM,CDH19,PRR5L,DAAM2,LOC101927967,PTGDS,LPAR1,SPP1,S100B,LOC100507336,SLC5A11,FAM107B,LOC100130370,ERBB3,TMEM144,ANLN,GPR37,VRK2,PMP22,APOD,RNF220,RGCC,CPM,PLA2G16,HEPACAM,PLD1,LDB3,DOCK1,CLMN,HEPN1,MBP,CNP,CLIC4,LINC00320,LINC00609,PIP4K2A,FRMD4B,CTNNA3,NCKAP5,QKI,CREB5,LINC01170,PLEKHH1,SIK3,LRP2,PPP2R2B,FGFR2,PCDH9,ELMO1,SLC44A1,PHLPP1,PDE4B,SLC24A2,ATP10B,GAB1,SCD,CDK18,DOCK10,PLCL1,PHLDB1,NINJ2,EDIL3,NDE1,MYO1E,IL1RAPL1,GLDN,MAP7,CAPN3,TCF12,SEPT7,TF,FMNL2,FRMD5,CRYAB,PXK,PDE8A,MEGF10,MAN2A1,FBXL7,TMEM165,FRYL,DLG1,DPYD,TTLL7,TMTC2,TRIM2,KIAA1598,GPRC5B,ERBB2IP,ZBTB20,GSN,DNAJC6,PTPRK,GATM,UNC5C,CA2,MAP4K4,ARAP2,PRUNE2,TJP1,HHIP,HAPLN2,CDH20,GPM6B,SYNJ2,USP54,PDE1C,SLAIN1,FUT8,DNM3,CLDND1,GRM3,PCSK6,LAMP2,HIPK2,WIPF1,ABCA2,APBB2,ATP8A1,ENOSF1,EFHD1,AGAP1,PICALM,MBNL2,HIP1,PREX1,SH3GL3,MARCH1,KIF13A,LPGAT1,FAXDC2,CNTN2,TSC22D4,APLP1,ZEB2,PIEZO2,MYO1D,COBL,SMA4,ZFHX4,PTN,FAM124A,ARHGAP21,SCD5,PEX5L,PTBP2,AMER2,MAP4K5,SLCO3A1,DIP2B,SH3D19,ZFYVE16,LANCL1,SORT1,FNBP1,CHD7,LOC101927768,PSEN1,RYBP,CBR1,FTH1,NEAT1,ADIPOR2,QDPR,TULP4,KLHL32,KLHL4,SUN2,CDK19,FAM13C,KIF6,SEMA6A,JAM3,RHOU,LOC100128079,KIF13B,HS3ST5,CHN2,SGK1,MTUS1,SEMA4D,PLXDC2,LOC100287225,PALM2,FOXN2,TESK2,NEO1,MOB3B,TUBA1A,KANK1,ATG4C,MARCKSL1,MVB12B,ACER3,AATK,IQGAP1,CUEDC1,SLC12A2,SLC22A15,CCP110,SECISBP2L,COLGALT2,SLC25A13,LRRC8D,SPATA6,PCDH9-AS2,RAD51B,GNG7,BIN1,YPEL2</t>
-        </is>
-      </c>
-      <c r="D26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Brain</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Tcell</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>ST18,PTPRC</t>
-        </is>
-      </c>
-      <c r="D27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Brain</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
           <t>VLMC</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>COLEC12,EBF1,IGFBP7,ITIH5,SLC6A12,MIR143HG,SLC12A7,NOTCH3,TXNIP,RERGL,GGT5,TBX2,TFPI,LEF1,BGN,IFITM1,COL1A2,IFITM3,MYL9,GPER1,COL6A2,FHL5,GNG11,LOC105377443,ATP1A2,CD9,EPAS1,TINAGL1,VIM,PTH1R,CFH,PDGFRB,SLC1A3,PRELP,SLC6A13,UACA,TGFBR2,SNTB1,SLC19A1,ADIRF,SLC38A11,GJC1,HIGD1B,AXL,DAAM2,NDUFA4L2,TNS1,COBLL1,LOC102467224,RHOJ,EPS8,SPARC,DCN,WDFY4,CPM,MFGE8,SMOC2,PTN,ABCA8,PALD1,MYO1B,RBPMS,ARHGAP29,ISYNA1,TRPC3,FAM65C,LAMA2,PTPRK,LHFP,DLC1,KANK3,ARHGAP42,ACSS3,CALD1,UTRN,HTR1F,PTGDS,MAML2,RGS5,SLC6A1,SLC20A2,GPC5,NR2F2-AS1,SLC30A10,RNF152,TNS2,RBMS3,KANK2,PDE7B,PRKG1,RCSD1,MYOF,B2M,SEMA5A,A2M,MCAM,YAP1,NID1,FN1,PLXDC1,MRC2,CA4,HES4,ETS1,PARD3,CDH6,ARHGAP10,PDE8B,GRM3,NR2F2,TJP1,ADGRF5,CLMN,CASC15,PLCB4,ARHGAP6,P2RY14,ZBTB20,RORA,PTEN,PDZD2,GRM8,COL4A3,LAMA4,LPP,TACC1,PLCE1,HSPB1,DACH1,DOCK1,ABCC9,ZFHX3,PDE8A,KIAA1109,APBB2,GRAMD3,COL4A4,ZEB1,MGLL,RNR2,TIMP3,KIRREL,FOXP1,TESC,CACHD1,ITGA1,FRZB,ZAK,ADAMTS9-AS2,LOC101927998,SH3RF1,FRMD3,AGRN,PRRX1,LAMC3,PHLDB2,CYTH3,LZTS1,NEAT1,GRK5,NBEAL1,SLC6A1-AS1,LGALS1,PARD3B,MPPED2,AKAP13,SLC12A2,PDE3A,SNRK,ECE1,SYNE2,C2CD2,PAG1,EFHD1,ATP6,GSN,DENND2A,CECR2,NFIA,CYTB,PREX2,CPE,DLEU2,COX3,PAPSS2,ACTB,UST,HLA-C,ANO3,LOC644135,CA2,FLNA,KIF13A,BCL2,SASH1,COX2,PIK3CD,HIP1,PLCL1,ST5,RHOB,ACTN4,FRMD6,BSG,ND3,PITPNM2,RNR1,ACTG1,COL6A1,EEF1DP3,CCDC3,ND1,ND4,ND2,LOC102724947,CPQ,ACTA2,H3F3B</t>
         </is>
       </c>
-      <c r="D28">
+      <c r="E26">
         <v>0</v>
       </c>
     </row>

</xml_diff>